<commit_message>
calc metrics for one-shot results with negative example
</commit_message>
<xml_diff>
--- a/src/results/llm/initial_testing_01/results_for_presentation_initial_testing.xlsx
+++ b/src/results/llm/initial_testing_01/results_for_presentation_initial_testing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\initial_testing_01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB674386-461F-4967-8463-5E7CA77FD6C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4620F94D-D1ED-43F7-A824-990DBC4A20B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="4" r:id="rId1"/>
@@ -289,7 +289,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -299,28 +299,27 @@
     <xf numFmtId="10" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -338,36 +337,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -657,7 +626,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E2F8CBD-665F-4514-96E7-546603B512CB}">
-  <dimension ref="A1:F65"/>
+  <dimension ref="A1:L65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" customWidth="1"/>
@@ -666,19 +635,23 @@
     <col min="4" max="4" width="17.140625" style="5" customWidth="1"/>
     <col min="5" max="5" width="13.7109375" style="5" customWidth="1"/>
     <col min="6" max="6" width="14.140625" style="5" customWidth="1"/>
+    <col min="10" max="10" width="23.7109375" customWidth="1"/>
+    <col min="11" max="11" width="23.85546875" customWidth="1"/>
+    <col min="12" max="12" width="21.5703125" customWidth="1"/>
+    <col min="14" max="14" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>0</v>
       </c>
@@ -698,7 +671,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
@@ -717,8 +690,11 @@
       <c r="F3" s="7">
         <v>0.56790237588980297</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J3" s="8"/>
+      <c r="K3" s="8"/>
+      <c r="L3" s="8"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>2</v>
       </c>
@@ -737,8 +713,11 @@
       <c r="F4" s="7">
         <v>0.60442987182720698</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>3</v>
       </c>
@@ -757,8 +736,11 @@
       <c r="F5" s="7">
         <v>0.59625862695241505</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>4</v>
       </c>
@@ -777,8 +759,11 @@
       <c r="F6" s="7">
         <v>0.67138435366112903</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>5</v>
       </c>
@@ -797,8 +782,11 @@
       <c r="F7" s="7">
         <v>0.320677619817825</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>6</v>
       </c>
@@ -817,8 +805,11 @@
       <c r="F8" s="7">
         <v>0.35685204527529601</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>7</v>
       </c>
@@ -837,8 +828,11 @@
       <c r="F9" s="7">
         <v>0.45795544598045201</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>8</v>
       </c>
@@ -857,8 +851,11 @@
       <c r="F10" s="7">
         <v>0.59339298647290994</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+    </row>
+    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>9</v>
       </c>
@@ -877,8 +874,11 @@
       <c r="F11" s="7">
         <v>0.53764768118497597</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J11" s="8"/>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>10</v>
       </c>
@@ -897,8 +897,11 @@
       <c r="F12" s="7">
         <v>0.57895655208515096</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J12" s="8"/>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>11</v>
       </c>
@@ -917,8 +920,11 @@
       <c r="F13" s="7">
         <v>0.60225374696568101</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+    </row>
+    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>12</v>
       </c>
@@ -937,8 +943,11 @@
       <c r="F14" s="7">
         <v>0.58985040711986303</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>13</v>
       </c>
@@ -957,8 +966,11 @@
       <c r="F15" s="7">
         <v>0.67202557967935905</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>14</v>
       </c>
@@ -977,8 +989,11 @@
       <c r="F16" s="7">
         <v>0.363630338245365</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>15</v>
       </c>
@@ -997,8 +1012,11 @@
       <c r="F17" s="7">
         <v>0.57960726468147805</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>51</v>
       </c>
@@ -1017,8 +1035,11 @@
       <c r="F18" s="7">
         <v>0.67550826272592501</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>52</v>
       </c>
@@ -1037,8 +1058,11 @@
       <c r="F19" s="6">
         <v>0.73632332330032302</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>53</v>
       </c>
@@ -1057,9 +1081,12 @@
       <c r="F20" s="7">
         <v>0.48988982228038302</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A21" s="9" t="s">
         <v>54</v>
       </c>
       <c r="B21" s="4">
@@ -1083,17 +1110,17 @@
         <v>0.73632332330032302</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A23" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="9"/>
-      <c r="C23" s="9"/>
-      <c r="D23" s="9"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="9"/>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>0</v>
       </c>
@@ -1113,7 +1140,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>1</v>
       </c>
@@ -1133,7 +1160,7 @@
         <v>0.41636436920596498</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>2</v>
       </c>
@@ -1153,7 +1180,7 @@
         <v>0.41339258660741302</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
         <v>3</v>
       </c>
@@ -1173,7 +1200,7 @@
         <v>0.40356564019448898</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>4</v>
       </c>
@@ -1193,7 +1220,7 @@
         <v>0.43446480424551898</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>5</v>
       </c>
@@ -1213,7 +1240,7 @@
         <v>0.25919801570897</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>6</v>
       </c>
@@ -1233,7 +1260,7 @@
         <v>0.290982336535481</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>7</v>
       </c>
@@ -1253,7 +1280,7 @@
         <v>0.36523517382413001</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>8</v>
       </c>
@@ -1474,7 +1501,7 @@
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
+      <c r="A43" s="9" t="s">
         <v>54</v>
       </c>
       <c r="B43" s="4">
@@ -1499,14 +1526,14 @@
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" s="9" t="s">
+      <c r="A45" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9"/>
-      <c r="D45" s="9"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="9"/>
+      <c r="B45" s="13"/>
+      <c r="C45" s="13"/>
+      <c r="D45" s="13"/>
+      <c r="E45" s="13"/>
+      <c r="F45" s="13"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="8" t="s">
@@ -1889,7 +1916,7 @@
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A65" s="14" t="s">
+      <c r="A65" s="9" t="s">
         <v>54</v>
       </c>
       <c r="B65" s="4">
@@ -1958,21 +1985,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+      <c r="N1" s="4"/>
+      <c r="O1" s="4"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -2422,14 +2449,14 @@
       <c r="I22" s="4"/>
     </row>
     <row r="24" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
+      <c r="B24" s="14"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
@@ -2852,14 +2879,14 @@
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" s="10" t="s">
+      <c r="A47" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B47" s="10"/>
-      <c r="C47" s="10"/>
-      <c r="D47" s="10"/>
-      <c r="E47" s="10"/>
-      <c r="F47" s="10"/>
+      <c r="B47" s="14"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="14"/>
+      <c r="E47" s="14"/>
+      <c r="F47" s="14"/>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
@@ -3323,16 +3350,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="F1" s="13" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="F1" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="13"/>
+      <c r="G1" s="12"/>
       <c r="I1" s="11" t="s">
         <v>46</v>
       </c>
@@ -3416,11 +3443,11 @@
         <v>0.60816326530612197</v>
       </c>
       <c r="C4" s="7">
-        <f t="shared" ref="C4:C22" si="0">B4-G4</f>
+        <f t="shared" ref="C4:C21" si="0">B4-G4</f>
         <v>-1.683673469387803E-2</v>
       </c>
       <c r="D4" s="7">
-        <f t="shared" ref="D4:D22" si="1">B4-M4</f>
+        <f t="shared" ref="D4:D21" si="1">B4-M4</f>
         <v>2.4829931972788932E-2</v>
       </c>
       <c r="F4" s="3" t="s">
@@ -4025,12 +4052,12 @@
       <c r="D22"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
@@ -4070,7 +4097,7 @@
         <v>0.79220779220779203</v>
       </c>
       <c r="C26" s="7">
-        <f t="shared" ref="C26:C44" si="2">B26-G4</f>
+        <f t="shared" ref="C26:C43" si="2">B26-G4</f>
         <v>0.16720779220779203</v>
       </c>
       <c r="D26" s="7">
@@ -4355,12 +4382,12 @@
       <c r="D44"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="12" t="s">
+      <c r="A45" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B45" s="12"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
@@ -4725,6 +4752,17 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C1:D1 C3:D21 C23:D23 C25:D43 C45:D45 C47:D65 C1591:D1048576">
+    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F2:F21">
     <cfRule type="colorScale" priority="53">
       <colorScale>
@@ -4747,6 +4785,38 @@
       </colorScale>
     </cfRule>
     <cfRule type="colorScale" priority="55">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G21">
+    <cfRule type="colorScale" priority="81">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="82">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="83">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4789,6 +4859,38 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J21">
+    <cfRule type="colorScale" priority="88">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="89">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="100"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="90">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L2:L21">
     <cfRule type="colorScale" priority="17">
       <colorScale>
@@ -4811,70 +4913,6 @@
       </colorScale>
     </cfRule>
     <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G21">
-    <cfRule type="colorScale" priority="81">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="82">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="100"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="83">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J21">
-    <cfRule type="colorScale" priority="88">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="89">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="100"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="90">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4917,17 +4955,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C1:D1 C25:D43 C3:D21 C47:D65 C23:D23 C45:D45 C1591:D1048576">
-    <cfRule type="cellIs" dxfId="0" priority="3" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="2" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="1" operator="equal">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
One-shot results to csv with json-repair
</commit_message>
<xml_diff>
--- a/src/results/llm/initial_testing_01/results_for_presentation_initial_testing.xlsx
+++ b/src/results/llm/initial_testing_01/results_for_presentation_initial_testing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\initial_testing_01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81240C69-8B45-404A-A16A-13B6E294F9FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D8FAB5-BC70-4C52-A0D0-653DA824C05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="15" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="4" r:id="rId1"/>
@@ -211,7 +211,7 @@
     <t>Using JSON-repair</t>
   </si>
   <si>
-    <t>JSON-repair (only one response for TASKS was previously unparsable)</t>
+    <t>JSON-repair (only one response for TASKS was previously unparsable - difference is visible in questions from Outlook to Relevance)</t>
   </si>
 </sst>
 </file>
@@ -309,12 +309,6 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -324,7 +318,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
@@ -658,40 +658,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="J1" s="15" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="E1" s="14"/>
+      <c r="F1" s="14"/>
+      <c r="J1" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="15"/>
-      <c r="O1" s="15"/>
+      <c r="K1" s="14"/>
+      <c r="L1" s="14"/>
+      <c r="M1" s="14"/>
+      <c r="N1" s="14"/>
+      <c r="O1" s="14"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="J2" s="10" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="13"/>
+      <c r="F2" s="13"/>
+      <c r="J2" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="10"/>
-      <c r="L2" s="10"/>
-      <c r="M2" s="10"/>
-      <c r="N2" s="10"/>
-      <c r="O2" s="10"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
@@ -1464,22 +1464,22 @@
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="10" t="s">
+      <c r="A24" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="J24" s="10" t="s">
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="J24" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="K24" s="10"/>
-      <c r="L24" s="10"/>
-      <c r="M24" s="10"/>
-      <c r="N24" s="10"/>
-      <c r="O24" s="10"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
@@ -2252,22 +2252,22 @@
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46" s="10" t="s">
+      <c r="A46" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B46" s="10"/>
-      <c r="C46" s="10"/>
-      <c r="D46" s="10"/>
-      <c r="E46" s="10"/>
-      <c r="F46" s="10"/>
-      <c r="J46" s="10" t="s">
+      <c r="B46" s="13"/>
+      <c r="C46" s="13"/>
+      <c r="D46" s="13"/>
+      <c r="E46" s="13"/>
+      <c r="F46" s="13"/>
+      <c r="J46" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="K46" s="10"/>
-      <c r="L46" s="10"/>
-      <c r="M46" s="10"/>
-      <c r="N46" s="10"/>
-      <c r="O46" s="10"/>
+      <c r="K46" s="13"/>
+      <c r="L46" s="13"/>
+      <c r="M46" s="13"/>
+      <c r="N46" s="13"/>
+      <c r="O46" s="13"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
@@ -3096,19 +3096,19 @@
     <col min="11" max="11" width="20.140625" style="5" customWidth="1"/>
     <col min="12" max="12" width="19" style="5" customWidth="1"/>
     <col min="13" max="13" width="17.28515625" style="5" customWidth="1"/>
-    <col min="14" max="14" width="15" style="5" customWidth="1"/>
+    <col min="14" max="14" width="19.28515625" style="5" customWidth="1"/>
     <col min="15" max="15" width="15.42578125" style="5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="15" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
       <c r="I1" s="16" t="s">
         <v>57</v>
       </c>
@@ -3119,22 +3119,22 @@
       <c r="N1" s="16"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="11"/>
-      <c r="C2" s="11"/>
-      <c r="D2" s="11"/>
-      <c r="E2" s="11"/>
-      <c r="F2" s="11"/>
-      <c r="I2" s="11" t="s">
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="I2" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="11"/>
-      <c r="K2" s="11"/>
-      <c r="L2" s="11"/>
-      <c r="M2" s="11"/>
-      <c r="N2" s="11"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="15"/>
       <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -3940,22 +3940,22 @@
       <c r="I24" s="2"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="11"/>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11"/>
-      <c r="E25" s="11"/>
-      <c r="F25" s="11"/>
-      <c r="I25" s="11" t="s">
+      <c r="B25" s="15"/>
+      <c r="C25" s="15"/>
+      <c r="D25" s="15"/>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
+      <c r="I25" s="15" t="s">
         <v>22</v>
       </c>
-      <c r="J25" s="11"/>
-      <c r="K25" s="11"/>
-      <c r="L25" s="11"/>
-      <c r="M25" s="11"/>
-      <c r="N25" s="11"/>
+      <c r="J25" s="15"/>
+      <c r="K25" s="15"/>
+      <c r="L25" s="15"/>
+      <c r="M25" s="15"/>
+      <c r="N25" s="15"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
@@ -4759,22 +4759,22 @@
       <c r="I47" s="2"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A48" s="11" t="s">
+      <c r="A48" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="B48" s="11"/>
-      <c r="C48" s="11"/>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="11"/>
-      <c r="I48" s="11" t="s">
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="I48" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="J48" s="11"/>
-      <c r="K48" s="11"/>
-      <c r="L48" s="11"/>
-      <c r="M48" s="11"/>
-      <c r="N48" s="11"/>
+      <c r="J48" s="15"/>
+      <c r="K48" s="15"/>
+      <c r="L48" s="15"/>
+      <c r="M48" s="15"/>
+      <c r="N48" s="15"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
@@ -5645,24 +5645,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="C1" s="12"/>
-      <c r="D1" s="12"/>
-      <c r="F1" s="14" t="s">
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="F1" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="14"/>
-      <c r="I1" s="13" t="s">
+      <c r="G1" s="12"/>
+      <c r="I1" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="13"/>
-      <c r="L1" s="13" t="s">
+      <c r="J1" s="11"/>
+      <c r="L1" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="13"/>
+      <c r="M1" s="11"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -6347,12 +6347,12 @@
       <c r="D22"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
+      <c r="B23" s="10"/>
+      <c r="C23" s="10"/>
+      <c r="D23" s="10"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
@@ -6677,12 +6677,12 @@
       <c r="D44"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="12" t="s">
+      <c r="A45" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B45" s="12"/>
-      <c r="C45" s="12"/>
-      <c r="D45" s="12"/>
+      <c r="B45" s="10"/>
+      <c r="C45" s="10"/>
+      <c r="D45" s="10"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
@@ -7037,6 +7037,42 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="A46:A65">
     <cfRule type="colorScale" priority="41">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B3:B21">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B25:B43">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B47:B65">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="percentile" val="50"/>
@@ -7250,42 +7286,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B3:B21">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B25:B43">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B47:B65">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="num" val="0"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="num" val="1"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sum up results for presentation
</commit_message>
<xml_diff>
--- a/src/results/llm/initial_testing_01/results_for_presentation_initial_testing.xlsx
+++ b/src/results/llm/initial_testing_01/results_for_presentation_initial_testing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\repos\Using-LLM-for-automated-feedback-generation-on-a-bachelor-thesis\src\results\llm\initial_testing_01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48D8FAB5-BC70-4C52-A0D0-653DA824C05E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17CE421D-88E4-4621-BE96-9E4B7364C077}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overall" sheetId="4" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="62">
   <si>
     <t>Model</t>
   </si>
@@ -213,6 +213,18 @@
   <si>
     <t>JSON-repair (only one response for TASKS was previously unparsable - difference is visible in questions from Outlook to Relevance)</t>
   </si>
+  <si>
+    <t>human1</t>
+  </si>
+  <si>
+    <t>human2</t>
+  </si>
+  <si>
+    <t>human3</t>
+  </si>
+  <si>
+    <t>F1 makro mēra vērtības</t>
+  </si>
 </sst>
 </file>
 
@@ -309,15 +321,6 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -328,6 +331,15 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -641,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E2F8CBD-665F-4514-96E7-546603B512CB}">
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:U66"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" customWidth="1"/>
@@ -655,45 +667,55 @@
     <col min="12" max="12" width="18" style="5" customWidth="1"/>
     <col min="13" max="13" width="17.28515625" style="5" customWidth="1"/>
     <col min="14" max="15" width="13.42578125" style="5" customWidth="1"/>
+    <col min="18" max="18" width="23.5703125" customWidth="1"/>
+    <col min="19" max="19" width="10.85546875" customWidth="1"/>
+    <col min="20" max="20" width="11.7109375" customWidth="1"/>
+    <col min="21" max="21" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A1" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="J1" s="14" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="J1" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14"/>
-      <c r="M1" s="14"/>
-      <c r="N1" s="14"/>
-      <c r="O1" s="14"/>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="13" t="s">
+      <c r="K1" s="11"/>
+      <c r="L1" s="11"/>
+      <c r="M1" s="11"/>
+      <c r="N1" s="11"/>
+      <c r="O1" s="11"/>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
-      <c r="J2" s="13" t="s">
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="J2" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="K2" s="13"/>
-      <c r="L2" s="13"/>
-      <c r="M2" s="13"/>
-      <c r="N2" s="13"/>
-      <c r="O2" s="13"/>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K2" s="10"/>
+      <c r="L2" s="10"/>
+      <c r="M2" s="10"/>
+      <c r="N2" s="10"/>
+      <c r="O2" s="10"/>
+      <c r="R2" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="S2" s="10"/>
+      <c r="T2" s="10"/>
+      <c r="U2" s="10"/>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
@@ -730,8 +752,18 @@
       <c r="O3" s="6" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R3" s="8"/>
+      <c r="S3" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="T3" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="U3" s="8" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
         <v>1</v>
       </c>
@@ -768,8 +800,20 @@
       <c r="O4" s="5">
         <v>0.56790237588980297</v>
       </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R4" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="S4" s="7">
+        <v>0.78304612706701404</v>
+      </c>
+      <c r="T4" s="7">
+        <v>0.69719032642402901</v>
+      </c>
+      <c r="U4" s="7">
+        <v>0.76954108569107804</v>
+      </c>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>2</v>
       </c>
@@ -806,8 +850,20 @@
       <c r="O5" s="5">
         <v>0.60388492181939202</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R5" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="S5" s="7">
+        <v>0.80147966804919502</v>
+      </c>
+      <c r="T5" s="7">
+        <v>0.69586147114953001</v>
+      </c>
+      <c r="U5" s="7">
+        <v>0.76385134456426296</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
         <v>3</v>
       </c>
@@ -844,8 +900,20 @@
       <c r="O6" s="5">
         <v>0.59943659412058703</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R6" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="S6" s="7">
+        <v>0.79962213225371104</v>
+      </c>
+      <c r="T6" s="7">
+        <v>0.69496220838286704</v>
+      </c>
+      <c r="U6" s="7">
+        <v>0.75782567947516399</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>4</v>
       </c>
@@ -882,8 +950,20 @@
       <c r="O7" s="5">
         <v>0.67138435366112903</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="S7" s="7">
+        <v>0.83331423242435398</v>
+      </c>
+      <c r="T7" s="7">
+        <v>0.69978773477687595</v>
+      </c>
+      <c r="U7" s="7">
+        <v>0.81241841580824603</v>
+      </c>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>5</v>
       </c>
@@ -920,8 +1000,20 @@
       <c r="O8" s="5">
         <v>0.320677619817825</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R8" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="S8" s="7">
+        <v>0.65352176886254798</v>
+      </c>
+      <c r="T8" s="7">
+        <v>0.62954963972810196</v>
+      </c>
+      <c r="U8" s="7">
+        <v>0.61177628027174302</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
         <v>6</v>
       </c>
@@ -958,8 +1050,20 @@
       <c r="O9" s="5">
         <v>0.35685204527529601</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R9" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="S9" s="7">
+        <v>0.67233886299511203</v>
+      </c>
+      <c r="T9" s="7">
+        <v>0.64547165310503796</v>
+      </c>
+      <c r="U9" s="7">
+        <v>0.63058194069840501</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
         <v>7</v>
       </c>
@@ -996,8 +1100,20 @@
       <c r="O10" s="5">
         <v>0.45795544598045201</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R10" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="S10" s="7">
+        <v>0.72811288880055602</v>
+      </c>
+      <c r="T10" s="7">
+        <v>0.68087875221514205</v>
+      </c>
+      <c r="U10" s="7">
+        <v>0.715714193164949</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
         <v>8</v>
       </c>
@@ -1034,8 +1150,20 @@
       <c r="O11" s="5">
         <v>0.59666144530428</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R11" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="S11" s="7">
+        <v>0.79656485033404401</v>
+      </c>
+      <c r="T11" s="7">
+        <v>0.69898798689479402</v>
+      </c>
+      <c r="U11" s="7">
+        <v>0.80123628745409903</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
         <v>9</v>
       </c>
@@ -1072,8 +1200,20 @@
       <c r="O12" s="5">
         <v>0.53764768118497597</v>
       </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R12" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="S12" s="7">
+        <v>0.76816976127320902</v>
+      </c>
+      <c r="T12" s="7">
+        <v>0.72033345689601502</v>
+      </c>
+      <c r="U12" s="7">
+        <v>0.73075718899403397</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>10</v>
       </c>
@@ -1110,8 +1250,20 @@
       <c r="O13" s="5">
         <v>0.57895655208515096</v>
       </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R13" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="S13" s="7">
+        <v>0.78814749780509197</v>
+      </c>
+      <c r="T13" s="7">
+        <v>0.73022739877981102</v>
+      </c>
+      <c r="U13" s="7">
+        <v>0.72333933531538297</v>
+      </c>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>11</v>
       </c>
@@ -1148,8 +1300,20 @@
       <c r="O14" s="5">
         <v>0.60225374696568101</v>
       </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R14" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="S14" s="7">
+        <v>0.80097603647286797</v>
+      </c>
+      <c r="T14" s="7">
+        <v>0.71417404174752996</v>
+      </c>
+      <c r="U14" s="7">
+        <v>0.75626690976063604</v>
+      </c>
+    </row>
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>12</v>
       </c>
@@ -1186,8 +1350,20 @@
       <c r="O15" s="5">
         <v>0.58985040711986303</v>
       </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R15" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="S15" s="7">
+        <v>0.79173076923076902</v>
+      </c>
+      <c r="T15" s="7">
+        <v>0.68994802392860599</v>
+      </c>
+      <c r="U15" s="7">
+        <v>0.80506388797208694</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>13</v>
       </c>
@@ -1224,8 +1400,20 @@
       <c r="O16" s="5">
         <v>0.67202557967935905</v>
       </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R16" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="S16" s="7">
+        <v>0.83596224212707804</v>
+      </c>
+      <c r="T16" s="6">
+        <v>0.77657591690481198</v>
+      </c>
+      <c r="U16" s="7">
+        <v>0.78122833990975704</v>
+      </c>
+    </row>
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>14</v>
       </c>
@@ -1262,8 +1450,20 @@
       <c r="O17" s="5">
         <v>0.36403791090493398</v>
       </c>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R17" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="S17" s="7">
+        <v>0.68161061557234903</v>
+      </c>
+      <c r="T17" s="7">
+        <v>0.63860852257918199</v>
+      </c>
+      <c r="U17" s="7">
+        <v>0.68117484636203596</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
         <v>15</v>
       </c>
@@ -1300,8 +1500,20 @@
       <c r="O18" s="5">
         <v>0.57960726468147805</v>
       </c>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R18" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="S18" s="7">
+        <v>0.789101252211315</v>
+      </c>
+      <c r="T18" s="7">
+        <v>0.69436241721353997</v>
+      </c>
+      <c r="U18" s="7">
+        <v>0.77605759066667002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
         <v>51</v>
       </c>
@@ -1338,8 +1550,20 @@
       <c r="O19" s="5">
         <v>0.67550826272592501</v>
       </c>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R19" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="S19" s="7">
+        <v>0.83743844753052399</v>
+      </c>
+      <c r="T19" s="7">
+        <v>0.76055460257203999</v>
+      </c>
+      <c r="U19" s="7">
+        <v>0.79254244103278504</v>
+      </c>
+    </row>
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
         <v>52</v>
       </c>
@@ -1376,8 +1600,20 @@
       <c r="O20" s="4">
         <v>0.74627587318398403</v>
       </c>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R20" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="S20" s="6">
+        <v>0.87275111483504597</v>
+      </c>
+      <c r="T20" s="7">
+        <v>0.76214905902143104</v>
+      </c>
+      <c r="U20" s="6">
+        <v>0.83914274034009595</v>
+      </c>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
         <v>53</v>
       </c>
@@ -1414,8 +1650,20 @@
       <c r="O21" s="5">
         <v>0.50695386702849299</v>
       </c>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="R21" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="S21" s="7">
+        <v>0.74782042940793703</v>
+      </c>
+      <c r="T21" s="7">
+        <v>0.71841346035966502</v>
+      </c>
+      <c r="U21" s="7">
+        <v>0.68078316629978497</v>
+      </c>
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
         <v>54</v>
       </c>
@@ -1463,25 +1711,25 @@
         <v>0.74627587318398403</v>
       </c>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A24" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="13"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="13"/>
-      <c r="E24" s="13"/>
-      <c r="F24" s="13"/>
-      <c r="J24" s="13" t="s">
+      <c r="B24" s="10"/>
+      <c r="C24" s="10"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="J24" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="13"/>
-      <c r="O24" s="13"/>
-    </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>0</v>
       </c>
@@ -1519,7 +1767,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
         <v>1</v>
       </c>
@@ -1557,7 +1805,7 @@
         <v>0.41636436920596498</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
         <v>2</v>
       </c>
@@ -1595,7 +1843,7 @@
         <v>0.41039878849066103</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>3</v>
       </c>
@@ -1633,7 +1881,7 @@
         <v>0.40368644926068398</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
         <v>4</v>
       </c>
@@ -1671,7 +1919,7 @@
         <v>0.43446480424551898</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
         <v>5</v>
       </c>
@@ -1709,7 +1957,7 @@
         <v>0.25919801570897</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
         <v>6</v>
       </c>
@@ -1747,7 +1995,7 @@
         <v>0.290982336535481</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>7</v>
       </c>
@@ -2252,22 +2500,22 @@
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A46" s="13" t="s">
+      <c r="A46" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B46" s="13"/>
-      <c r="C46" s="13"/>
-      <c r="D46" s="13"/>
-      <c r="E46" s="13"/>
-      <c r="F46" s="13"/>
-      <c r="J46" s="13" t="s">
+      <c r="B46" s="10"/>
+      <c r="C46" s="10"/>
+      <c r="D46" s="10"/>
+      <c r="E46" s="10"/>
+      <c r="F46" s="10"/>
+      <c r="J46" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="K46" s="13"/>
-      <c r="L46" s="13"/>
-      <c r="M46" s="13"/>
-      <c r="N46" s="13"/>
-      <c r="O46" s="13"/>
+      <c r="K46" s="10"/>
+      <c r="L46" s="10"/>
+      <c r="M46" s="10"/>
+      <c r="N46" s="10"/>
+      <c r="O46" s="10"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
@@ -3040,7 +3288,8 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
+    <mergeCell ref="R2:U2"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A24:F24"/>
     <mergeCell ref="A46:F46"/>
@@ -3051,7 +3300,7 @@
     <mergeCell ref="J1:O1"/>
   </mergeCells>
   <conditionalFormatting sqref="B2:F1048576">
-    <cfRule type="colorScale" priority="2">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="percentile" val="50"/>
@@ -3063,7 +3312,55 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:O66">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S4:S21">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S1:U1048576">
     <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T4:T21">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="num" val="0"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="num" val="1"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U4:U21">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0"/>
         <cfvo type="percentile" val="50"/>
@@ -3101,40 +3398,40 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="I1" s="16" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="I1" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="16"/>
-      <c r="L1" s="16"/>
-      <c r="M1" s="16"/>
-      <c r="N1" s="16"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+      <c r="L1" s="13"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="13"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-      <c r="D2" s="15"/>
-      <c r="E2" s="15"/>
-      <c r="F2" s="15"/>
-      <c r="I2" s="15" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="I2" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="15"/>
-      <c r="K2" s="15"/>
-      <c r="L2" s="15"/>
-      <c r="M2" s="15"/>
-      <c r="N2" s="15"/>
+      <c r="J2" s="12"/>
+      <c r="K2" s="12"/>
+      <c r="L2" s="12"/>
+      <c r="M2" s="12"/>
+      <c r="N2" s="12"/>
       <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
@@ -3940,22 +4237,22 @@
       <c r="I24" s="2"/>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A25" s="15" t="s">
+      <c r="A25" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="15"/>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="I25" s="15" t="s">
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="I25" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15"/>
-      <c r="L25" s="15"/>
-      <c r="M25" s="15"/>
-      <c r="N25" s="15"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
@@ -4759,22 +5056,22 @@
       <c r="I47" s="2"/>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A48" s="15" t="s">
+      <c r="A48" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="B48" s="15"/>
-      <c r="C48" s="15"/>
-      <c r="D48" s="15"/>
-      <c r="E48" s="15"/>
-      <c r="F48" s="15"/>
-      <c r="I48" s="15" t="s">
+      <c r="B48" s="12"/>
+      <c r="C48" s="12"/>
+      <c r="D48" s="12"/>
+      <c r="E48" s="12"/>
+      <c r="F48" s="12"/>
+      <c r="I48" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="J48" s="15"/>
-      <c r="K48" s="15"/>
-      <c r="L48" s="15"/>
-      <c r="M48" s="15"/>
-      <c r="N48" s="15"/>
+      <c r="J48" s="12"/>
+      <c r="K48" s="12"/>
+      <c r="L48" s="12"/>
+      <c r="M48" s="12"/>
+      <c r="N48" s="12"/>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
@@ -5645,24 +5942,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="10" t="s">
+      <c r="A1" s="14" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="F1" s="12" t="s">
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
+      <c r="F1" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="G1" s="12"/>
-      <c r="I1" s="11" t="s">
+      <c r="G1" s="16"/>
+      <c r="I1" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="J1" s="11"/>
-      <c r="L1" s="11" t="s">
+      <c r="J1" s="15"/>
+      <c r="L1" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="M1" s="11"/>
+      <c r="M1" s="15"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
@@ -6347,12 +6644,12 @@
       <c r="D22"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
@@ -6677,12 +6974,12 @@
       <c r="D44"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="10" t="s">
+      <c r="A45" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B45" s="10"/>
-      <c r="C45" s="10"/>
-      <c r="D45" s="10"/>
+      <c r="B45" s="14"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">

</xml_diff>